<commit_message>
Update pilot import file
</commit_message>
<xml_diff>
--- a/imports/zid_import_pilot.xlsx
+++ b/imports/zid_import_pilot.xlsx
@@ -1464,7 +1464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DH17"/>
+  <dimension ref="A1:DH16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="17" customWidth="1" style="47" min="1" max="1"/>
@@ -2515,12 +2515,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>طقم فحمات فرامل امامية هونداي النترا 2016-2020</t>
+          <t>طقم فحمات فرامل امامية هونداي النترا 2016-2020 (58101F2A00)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Front Brake Pad Kit Hyundai Elantra 2016-2020</t>
+          <t>Front Brake Pad Kit Hyundai Elantra 2016-2020 (58101F2A00)</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -2559,27 +2559,27 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>58101F2A00, طقم فحمات فرامل امامية هونداي النترا 2016-2020, Front Brake Pad Kit Hyundai Elantra 2016-2020</t>
+          <t>58101F2A00, طقم فحمات فرامل امامية هونداي النترا 2016-2020 (58101F2A00), Front Brake Pad Kit Hyundai Elantra 2016-2020 (58101F2A00)</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>&lt;p&gt;طقم فحمات فرامل امامية هونداي النترا 2016-2020.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;رقم القطعة: 58101F2A00&lt;/li&gt;&lt;li&gt;النوع المتوفر: بديل (تجاري)&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;السيارات المتوافقة&lt;/h3&gt;&lt;table&gt;&lt;thead&gt;&lt;tr&gt;&lt;th&gt;الشركة&lt;/th&gt;&lt;th&gt;الموديل&lt;/th&gt;&lt;th&gt;سنوات الصنع&lt;/th&gt;&lt;/tr&gt;&lt;/thead&gt;&lt;tbody&gt;&lt;tr&gt;&lt;td&gt;هونداي&lt;/td&gt;&lt;td&gt;النترا&lt;/td&gt;&lt;td&gt;2016-2020&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;&lt;p&gt;نتحقق من توافق القطعة مع سيارتك برقم الهيكل (VIN). أرسل رقم الهيكل (VIN) عبر واتساب ونؤكد لك القطعة قبل الشحن.&lt;/p&gt;</t>
+          <t>&lt;p&gt;طقم فحمات فرامل امامية هونداي النترا 2016-2020 (58101F2A00).&lt;/p&gt;&lt;ul&gt;&lt;li&gt;رقم القطعة: 58101F2A00&lt;/li&gt;&lt;li&gt;النوع المتوفر: بديل (تجاري)&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;السيارات المتوافقة&lt;/h3&gt;&lt;table&gt;&lt;thead&gt;&lt;tr&gt;&lt;th&gt;الشركة&lt;/th&gt;&lt;th&gt;الموديل&lt;/th&gt;&lt;th&gt;سنوات الصنع&lt;/th&gt;&lt;/tr&gt;&lt;/thead&gt;&lt;tbody&gt;&lt;tr&gt;&lt;td&gt;هونداي&lt;/td&gt;&lt;td&gt;النترا&lt;/td&gt;&lt;td&gt;2016-2020&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;&lt;p&gt;نتحقق من توافق القطعة مع سيارتك برقم الهيكل (VIN). أرسل رقم الهيكل (VIN) عبر واتساب ونؤكد لك القطعة قبل الشحن.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Front Brake Pad Kit Hyundai Elantra 2016-2020.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Part number: 58101F2A00&lt;/li&gt;&lt;li&gt;Available as: Aftermarket&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Compatible vehicles&lt;/h3&gt;&lt;table&gt;&lt;thead&gt;&lt;tr&gt;&lt;th&gt;Make&lt;/th&gt;&lt;th&gt;Model&lt;/th&gt;&lt;th&gt;Years&lt;/th&gt;&lt;/tr&gt;&lt;/thead&gt;&lt;tbody&gt;&lt;tr&gt;&lt;td&gt;Hyundai&lt;/td&gt;&lt;td&gt;Elantra&lt;/td&gt;&lt;td&gt;2016-2020&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;&lt;p&gt;We check the part fits your car by VIN. Send your VIN on WhatsApp and we'll confirm the part before shipping.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Front Brake Pad Kit Hyundai Elantra 2016-2020 (58101F2A00).&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Part number: 58101F2A00&lt;/li&gt;&lt;li&gt;Available as: Aftermarket&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Compatible vehicles&lt;/h3&gt;&lt;table&gt;&lt;thead&gt;&lt;tr&gt;&lt;th&gt;Make&lt;/th&gt;&lt;th&gt;Model&lt;/th&gt;&lt;th&gt;Years&lt;/th&gt;&lt;/tr&gt;&lt;/thead&gt;&lt;tbody&gt;&lt;tr&gt;&lt;td&gt;Hyundai&lt;/td&gt;&lt;td&gt;Elantra&lt;/td&gt;&lt;td&gt;2016-2020&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;&lt;p&gt;We check the part fits your car by VIN. Send your VIN on WhatsApp and we'll confirm the part before shipping.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>طقم فحمات فرامل امامية هونداي النترا 2016-2020</t>
+          <t>طقم فحمات فرامل امامية هونداي النترا 2016-2020 (58101F2A00)</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>Front Brake Pad Kit Hyundai Elantra 2016-2020</t>
+          <t>Front Brake Pad Kit Hyundai Elantra 2016-2020 (58101F2A00)</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
@@ -2968,21 +2968,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>353102G300</t>
+          <t>5221760010</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>INJECTOR ASSY-FUEL هونداي سوناتا 2011-2014</t>
+          <t>مسمار تويوتا لاند كروزر 1998-2006</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>INJECTOR ASSY-FUEL Hyundai Sonata 2011-2014</t>
+          <t>BOLT, BODY MOUNTING Toyota Land Cruiser 1998-2006</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>81</v>
+        <v>149</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -2996,15 +2996,19 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>تسوق حسب السيارة &gt; هونداي, تسوق حسب السيارة &gt; هونداي &gt; هونداي سوناتا, تسوق حسب القسم &gt; قطع متنوعة</t>
+          <t>تسوق حسب السيارة &gt; تويوتا, تسوق حسب السيارة &gt; تويوتا &gt; تويوتا لاند كروزر, تسوق حسب القسم &gt; قطع متنوعة</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Shop by Vehicle &gt; Hyundai, Shop by Vehicle &gt; Hyundai &gt; Hyundai Sonata, Shop by Category &gt; Other Parts</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr"/>
+          <t>Shop by Vehicle &gt; Toyota, Shop by Vehicle &gt; Toyota &gt; Toyota Land Cruiser, Shop by Category &gt; Other Parts</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Mo-ai-sys/autospace-part-images/main/parts/5221760010_1.jpg, https://raw.githubusercontent.com/Mo-ai-sys/autospace-part-images/main/parts/5221760010_2.jpg</t>
+        </is>
+      </c>
       <c r="R15" t="inlineStr">
         <is>
           <t>No</t>
@@ -3017,27 +3021,27 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>353102G300, INJECTOR ASSY-FUEL هونداي سوناتا 2011-2014, INJECTOR ASSY-FUEL Hyundai Sonata 2011-2014</t>
+          <t>5221760010, مسمار تويوتا لاند كروزر 1998-2006, BOLT, BODY MOUNTING Toyota Land Cruiser 1998-2006</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>&lt;p&gt;INJECTOR ASSY-FUEL هونداي سوناتا 2011-2014.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;رقم القطعة: 353102G300&lt;/li&gt;&lt;li&gt;النوع المتوفر: أصلي (وكالة) / بديل (تجاري)&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;السيارات المتوافقة&lt;/h3&gt;&lt;table&gt;&lt;thead&gt;&lt;tr&gt;&lt;th&gt;الشركة&lt;/th&gt;&lt;th&gt;الموديل&lt;/th&gt;&lt;th&gt;سنوات الصنع&lt;/th&gt;&lt;/tr&gt;&lt;/thead&gt;&lt;tbody&gt;&lt;tr&gt;&lt;td&gt;هونداي&lt;/td&gt;&lt;td&gt;سوناتا&lt;/td&gt;&lt;td&gt;2011-2014&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;&lt;p&gt;نتحقق من توافق القطعة مع سيارتك برقم الهيكل (VIN). أرسل رقم الهيكل (VIN) عبر واتساب ونؤكد لك القطعة قبل الشحن.&lt;/p&gt;</t>
+          <t>&lt;p&gt;مسمار تويوتا لاند كروزر 1998-2006.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;رقم القطعة: 5221760010&lt;/li&gt;&lt;li&gt;النوع المتوفر: أصلي (وكالة)&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;السيارات المتوافقة&lt;/h3&gt;&lt;table&gt;&lt;thead&gt;&lt;tr&gt;&lt;th&gt;الشركة&lt;/th&gt;&lt;th&gt;الموديل&lt;/th&gt;&lt;th&gt;سنوات الصنع&lt;/th&gt;&lt;/tr&gt;&lt;/thead&gt;&lt;tbody&gt;&lt;tr&gt;&lt;td&gt;تويوتا&lt;/td&gt;&lt;td&gt;لاند كروزر&lt;/td&gt;&lt;td&gt;1998-2002&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;تويوتا&lt;/td&gt;&lt;td&gt;لاند كروزر&lt;/td&gt;&lt;td&gt;1998-2006&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;&lt;p&gt;نتحقق من توافق القطعة مع سيارتك برقم الهيكل (VIN). أرسل رقم الهيكل (VIN) عبر واتساب ونؤكد لك القطعة قبل الشحن.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>&lt;p&gt;INJECTOR ASSY-FUEL Hyundai Sonata 2011-2014.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Part number: 353102G300&lt;/li&gt;&lt;li&gt;Available as: Genuine (OEM) / Aftermarket&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Compatible vehicles&lt;/h3&gt;&lt;table&gt;&lt;thead&gt;&lt;tr&gt;&lt;th&gt;Make&lt;/th&gt;&lt;th&gt;Model&lt;/th&gt;&lt;th&gt;Years&lt;/th&gt;&lt;/tr&gt;&lt;/thead&gt;&lt;tbody&gt;&lt;tr&gt;&lt;td&gt;Hyundai&lt;/td&gt;&lt;td&gt;Sonata&lt;/td&gt;&lt;td&gt;2011-2014&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;&lt;p&gt;We check the part fits your car by VIN. Send your VIN on WhatsApp and we'll confirm the part before shipping.&lt;/p&gt;</t>
+          <t>&lt;p&gt;BOLT, BODY MOUNTING Toyota Land Cruiser 1998-2006.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Part number: 5221760010&lt;/li&gt;&lt;li&gt;Available as: Genuine (OEM)&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Compatible vehicles&lt;/h3&gt;&lt;table&gt;&lt;thead&gt;&lt;tr&gt;&lt;th&gt;Make&lt;/th&gt;&lt;th&gt;Model&lt;/th&gt;&lt;th&gt;Years&lt;/th&gt;&lt;/tr&gt;&lt;/thead&gt;&lt;tbody&gt;&lt;tr&gt;&lt;td&gt;Toyota&lt;/td&gt;&lt;td&gt;Land Cruiser&lt;/td&gt;&lt;td&gt;1998-2002&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Toyota&lt;/td&gt;&lt;td&gt;Land Cruiser&lt;/td&gt;&lt;td&gt;1998-2006&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;&lt;p&gt;We check the part fits your car by VIN. Send your VIN on WhatsApp and we'll confirm the part before shipping.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>INJECTOR ASSY-FUEL هونداي سوناتا 2011-2014</t>
+          <t>مسمار تويوتا لاند كروزر 1998-2006</t>
         </is>
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>INJECTOR ASSY-FUEL Hyundai Sonata 2011-2014</t>
+          <t>BOLT, BODY MOUNTING Toyota Land Cruiser 1998-2006</t>
         </is>
       </c>
       <c r="AH15" t="inlineStr">
@@ -3067,23 +3071,23 @@
       </c>
       <c r="CW15" t="inlineStr">
         <is>
-          <t>2011, 2012, 2013, 2014</t>
+          <t>1998, 1999, 2000, 2001, 2002, 2003, 2004, 2005, 2006</t>
         </is>
       </c>
       <c r="CX15" t="inlineStr">
         <is>
-          <t>2011, 2012, 2013, 2014</t>
+          <t>1998, 1999, 2000, 2001, 2002, 2003, 2004, 2005, 2006</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>353102G300-ORIG</t>
+          <t>5221760010-ORIG</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>362</v>
+        <v>149</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3098,31 +3102,6 @@
       <c r="AL16" t="inlineStr">
         <is>
           <t>Genuine (OEM)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>353102G300-REPL</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>81</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>infinite</t>
-        </is>
-      </c>
-      <c r="AK17" t="inlineStr">
-        <is>
-          <t>بديل (تجاري)</t>
-        </is>
-      </c>
-      <c r="AL17" t="inlineStr">
-        <is>
-          <t>Aftermarket</t>
         </is>
       </c>
     </row>

</xml_diff>